<commit_message>
docs: clarify bulk-import template with better examples
Replaces the example rows with a progression that demonstrates all three
cases: no alternatives (blank cell), a single alternative, and multiple
alternatives separated by ';'. Adds a notes section below the examples
explaining the semicolon separator rule.

Notes live only in column A so the import parser (which requires both
front and back to be non-empty) safely ignores them if the user forgets
to delete them before uploading.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Flashcards_Template.xlsx
+++ b/public/Flashcards_Template.xlsx
@@ -1,37 +1,127 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Flashcards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Flashcards" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>Front (Prompt)</t>
+  </si>
+  <si>
+    <t>Back (Target Answer)</t>
+  </si>
+  <si>
+    <t>Accepted Answers</t>
+  </si>
+  <si>
+    <t>What is the powerhouse of the cell?</t>
+  </si>
+  <si>
+    <t>Mitochondria</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>What is the capital of France?</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>paris</t>
+  </si>
+  <si>
+    <t>What is another name for a heart attack?</t>
+  </si>
+  <si>
+    <t>Myocardial Infarction</t>
+  </si>
+  <si>
+    <t>Heart Attack; MI; Acute MI; AMI</t>
+  </si>
+  <si>
+    <t>What classification system is used for male pattern baldness?</t>
+  </si>
+  <si>
+    <t>Hamilton-Norwood</t>
+  </si>
+  <si>
+    <t>Norwood Scale; Norwood; Hamilton Scale</t>
+  </si>
+  <si>
+    <t>NOTES — how to fill this template</t>
+  </si>
+  <si>
+    <t>1. 'Front (Prompt)' and 'Back (Target Answer)' are required. 'Accepted Answers' is optional.</t>
+  </si>
+  <si>
+    <t>2. To add MORE THAN ONE alternative, put them in a single cell separated by a semicolon ';'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Example: 'Heart Attack; MI; Acute MI; AMI'  =&gt;  creates a card that accepts all four as correct.</t>
+  </si>
+  <si>
+    <t>3. Use a semicolon ';', NOT a comma. Commas inside an answer (e.g. 'Addison's disease, primary') will NOT be split.</t>
+  </si>
+  <si>
+    <t>4. Leading/trailing spaces around each alternative are fine — they are trimmed automatically.</t>
+  </si>
+  <si>
+    <t>5. Leave 'Accepted Answers' blank if a card has no alternatives (row 2 above is an example).</t>
+  </si>
+  <si>
+    <t>6. Delete these notes and the example rows before uploading your own cards.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <color rgb="FFA3A3A3"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9C111"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF262626"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,81 +136,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -199,6 +241,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -233,6 +276,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -267,20 +311,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -402,77 +442,157 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Front (Prompt)</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Back (Target Answer)</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Accepted Answers</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>What is the powerhouse of the cell?</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Mitochondria</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mitochondrion</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>What classification system is used for male pattern baldness?</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Hamilton-Norwood</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Norwood Scale; Norwood</t>
-        </is>
+    <row r="1" ht="22" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: keep only multi-alternative examples in bulk-import template
Removes the two simpler example rows so the template focuses on the
pattern users most commonly stumble on — separating multiple accepted
answers with semicolons.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Flashcards_Template.xlsx
+++ b/public/Flashcards_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Front (Prompt)</t>
   </si>
@@ -22,24 +22,6 @@
     <t>Accepted Answers</t>
   </si>
   <si>
-    <t>What is the powerhouse of the cell?</t>
-  </si>
-  <si>
-    <t>Mitochondria</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>What is the capital of France?</t>
-  </si>
-  <si>
-    <t>Paris</t>
-  </si>
-  <si>
-    <t>paris</t>
-  </si>
-  <si>
     <t>What is another name for a heart attack?</t>
   </si>
   <si>
@@ -76,7 +58,7 @@
     <t>4. Leading/trailing spaces around each alternative are fine — they are trimmed automatically.</t>
   </si>
   <si>
-    <t>5. Leave 'Accepted Answers' blank if a card has no alternatives (row 2 above is an example).</t>
+    <t>5. Leave 'Accepted Answers' blank if a card has no alternatives.</t>
   </si>
   <si>
     <t>6. Delete these notes and the example rows before uploading your own cards.</t>
@@ -488,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -529,66 +511,44 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="5" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="6" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+    </row>
+    <row r="7" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: split bulk-import template into data + instructions sheets
Sheet 1 "Flashcards" now holds only the header row and two example
cards, keeping the workspace uncluttered for users pasting in hundreds
of rows at once. Sheet 2 "Instructions" holds the full how-to guide.

The uploader already reads only worksheets[0], so Sheet 2 is safely
ignored. Added a comment to BulkImportCards.tsx so that behavior stays
intentional.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Flashcards_Template.xlsx
+++ b/public/Flashcards_Template.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Flashcards" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Front (Prompt)</t>
   </si>
@@ -40,35 +41,71 @@
     <t>Norwood Scale; Norwood; Hamilton Scale</t>
   </si>
   <si>
-    <t>NOTES — how to fill this template</t>
-  </si>
-  <si>
-    <t>1. 'Front (Prompt)' and 'Back (Target Answer)' are required. 'Accepted Answers' is optional.</t>
-  </si>
-  <si>
-    <t>2. To add MORE THAN ONE alternative, put them in a single cell separated by a semicolon ';'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Example: 'Heart Attack; MI; Acute MI; AMI'  =&gt;  creates a card that accepts all four as correct.</t>
-  </si>
-  <si>
-    <t>3. Use a semicolon ';', NOT a comma. Commas inside an answer (e.g. 'Addison's disease, primary') will NOT be split.</t>
-  </si>
-  <si>
-    <t>4. Leading/trailing spaces around each alternative are fine — they are trimmed automatically.</t>
-  </si>
-  <si>
-    <t>5. Leave 'Accepted Answers' blank if a card has no alternatives.</t>
-  </si>
-  <si>
-    <t>6. Delete these notes and the example rows before uploading your own cards.</t>
+    <t>How to fill in the Flashcards sheet</t>
+  </si>
+  <si>
+    <t>Only the first sheet ("Flashcards") is imported. This sheet is for reference and is ignored by the uploader, so you can leave it alone.</t>
+  </si>
+  <si>
+    <t>REQUIRED vs OPTIONAL COLUMNS</t>
+  </si>
+  <si>
+    <t>• Front (Prompt)  — required. The question or cue shown on the front of the card.</t>
+  </si>
+  <si>
+    <t>• Back (Target Answer)  — required. The primary correct answer.</t>
+  </si>
+  <si>
+    <t>• Accepted Answers  — optional. Other wordings that should also count as correct.</t>
+  </si>
+  <si>
+    <t>ADDING MULTIPLE ALTERNATIVE ANSWERS</t>
+  </si>
+  <si>
+    <t>Put all alternatives in a single cell, separated by a semicolon ';'.</t>
+  </si>
+  <si>
+    <t>Example:  Heart Attack; MI; Acute MI; AMI   →  the card accepts all four as correct.</t>
+  </si>
+  <si>
+    <t>SEMICOLONS vs COMMAS</t>
+  </si>
+  <si>
+    <t>Use ';' — NOT ','. Commas inside an answer (e.g. "Addison's disease, primary") are left untouched.</t>
+  </si>
+  <si>
+    <t>OTHER RULES</t>
+  </si>
+  <si>
+    <t>• Leading/trailing spaces around each alternative are trimmed automatically.</t>
+  </si>
+  <si>
+    <t>• Leave 'Accepted Answers' blank if a card has no alternatives.</t>
+  </si>
+  <si>
+    <t>• You can delete the two example rows before uploading your own cards.</t>
+  </si>
+  <si>
+    <t>• You can paste up to ~500 rows per upload without issue.</t>
+  </si>
+  <si>
+    <t>COMMON MISTAKES</t>
+  </si>
+  <si>
+    <t>• Putting each alternative in its own cell — the uploader only reads columns A, B, C.</t>
+  </si>
+  <si>
+    <t>• Using "|" or "/" as a separator — only ";" is supported.</t>
+  </si>
+  <si>
+    <t>• Adding a 4th column — extra columns are ignored.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -83,12 +120,25 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="14"/>
     </font>
     <font>
       <color rgb="FFA3A3A3"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -98,11 +148,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF9C111"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF262626"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -126,9 +171,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -511,44 +566,118 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="3" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="5" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="6" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="7" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+    <row r="8" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="10" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+    <row r="11" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>